<commit_message>
updated excel data file
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="98">
   <si>
     <t xml:space="preserve">My Data, My Code</t>
   </si>
@@ -236,19 +236,37 @@
     <t xml:space="preserve">travel was tiring study was shorter than usual</t>
   </si>
   <si>
+    <t xml:space="preserve">Learning c++</t>
+  </si>
+  <si>
     <t xml:space="preserve">Did a short study session despite low energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preparing for ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Working on communication skills</t>
   </si>
   <si>
     <t xml:space="preserve">weekend routine was mostly reset, tv and phone</t>
   </si>
   <si>
+    <t xml:space="preserve">Enjoy fresher party</t>
+  </si>
+  <si>
     <t xml:space="preserve">Travel was tiring, study was shorter than usual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work on error and debugging on the project</t>
   </si>
   <si>
     <t xml:space="preserve">high</t>
   </si>
   <si>
     <t xml:space="preserve">classe travel took a lot of time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Making project Report</t>
   </si>
   <si>
     <t xml:space="preserve">neutral</t>
@@ -266,13 +284,37 @@
     <t xml:space="preserve">Excellent</t>
   </si>
   <si>
+    <t xml:space="preserve">Build function and more project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restless</t>
+  </si>
+  <si>
     <t xml:space="preserve">unsatisfied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">packaging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feeling tired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lonely</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leaving home</t>
   </si>
   <si>
     <t xml:space="preserve">stressed</t>
   </si>
   <si>
-    <t xml:space="preserve">Reg</t>
+    <t xml:space="preserve">Do corrections  in project and project completed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exploring university</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shopping</t>
   </si>
 </sst>
 </file>
@@ -1863,7 +1905,7 @@
         <v>54</v>
       </c>
       <c r="N21" s="18" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1951,7 +1993,7 @@
         <v>56</v>
       </c>
       <c r="N23" s="18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1995,10 +2037,10 @@
         <v>56</v>
       </c>
       <c r="N24" s="18" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="n">
         <v>46266</v>
       </c>
@@ -2039,7 +2081,7 @@
         <v>56</v>
       </c>
       <c r="N25" s="18" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2083,7 +2125,7 @@
         <v>61</v>
       </c>
       <c r="N26" s="18" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2127,7 +2169,7 @@
         <v>56</v>
       </c>
       <c r="N27" s="18" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2171,10 +2213,10 @@
         <v>56</v>
       </c>
       <c r="N28" s="18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="n">
         <v>46270</v>
       </c>
@@ -2215,7 +2257,7 @@
         <v>56</v>
       </c>
       <c r="N29" s="18" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2256,10 +2298,10 @@
         <v>53</v>
       </c>
       <c r="M30" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N30" s="18" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2303,7 +2345,7 @@
         <v>56</v>
       </c>
       <c r="N31" s="18" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2338,16 +2380,16 @@
         <v>530</v>
       </c>
       <c r="K32" s="17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="L32" s="17" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="M32" s="17" t="s">
         <v>61</v>
       </c>
       <c r="N32" s="18" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2385,7 +2427,7 @@
         <v>52</v>
       </c>
       <c r="L33" s="17" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="M33" s="17" t="s">
         <v>56</v>
@@ -2426,7 +2468,7 @@
         <v>265</v>
       </c>
       <c r="K34" s="17" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="L34" s="17" t="s">
         <v>53</v>
@@ -2473,13 +2515,13 @@
         <v>52</v>
       </c>
       <c r="L35" s="17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="M35" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N35" s="18" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2517,13 +2559,13 @@
         <v>52</v>
       </c>
       <c r="L36" s="17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="M36" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N36" s="18" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2611,7 +2653,7 @@
         <v>56</v>
       </c>
       <c r="N38" s="18" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2649,13 +2691,13 @@
         <v>52</v>
       </c>
       <c r="L39" s="17" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="M39" s="17" t="s">
         <v>56</v>
       </c>
       <c r="N39" s="18" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2699,7 +2741,7 @@
         <v>61</v>
       </c>
       <c r="N40" s="18" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2743,7 +2785,7 @@
         <v>61</v>
       </c>
       <c r="N41" s="18" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2781,13 +2823,13 @@
         <v>52</v>
       </c>
       <c r="L42" s="17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="M42" s="17" t="s">
         <v>56</v>
       </c>
       <c r="N42" s="18" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2866,7 +2908,7 @@
         <v>510</v>
       </c>
       <c r="K44" s="17" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="L44" s="17" t="s">
         <v>53</v>
@@ -2878,7 +2920,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="n">
         <v>46286</v>
       </c>
@@ -2910,16 +2952,16 @@
         <v>540</v>
       </c>
       <c r="K45" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="L45" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="L45" s="17" t="s">
-        <v>76</v>
-      </c>
       <c r="M45" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N45" s="18" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2998,16 +3040,16 @@
         <v>540</v>
       </c>
       <c r="K47" s="17" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="L47" s="17" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="M47" s="17" t="s">
         <v>56</v>
       </c>
       <c r="N47" s="18" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3051,7 +3093,7 @@
         <v>56</v>
       </c>
       <c r="N48" s="18" t="s">
-        <v>65</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="25.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3089,13 +3131,13 @@
         <v>52</v>
       </c>
       <c r="L49" s="17" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="M49" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N49" s="18" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>